<commit_message>
Expand isolated UI and auth API tests
</commit_message>
<xml_diff>
--- a/_testing/test_cases.xlsx
+++ b/_testing/test_cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -701,8 +701,309 @@
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>API-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NID API</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NID verification rejects a missing payload</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>API tests run against a disposable, seeded SQLite database.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>POST an empty JSON object to /api/auth/verify-nid.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>HTTP 400 with a validation error; no records are created.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>API-002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NID API</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NID verification rejects an invalid NID format</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>API tests run against a disposable, seeded SQLite database.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Submit a short NID with a date of birth.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>HTTP 400 with an NID format validation error.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>API-003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NID API</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NID verification accepts a valid unregistered mock NID</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mock NID verification is used; only the temporary database is queried.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Submit a valid 10-digit NID and date of birth.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HTTP 200, verified identity data, and alreadyRegistered=false.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>API-004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NID API</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NID verification detects an existing seeded account</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Temporary test database contains the documented demo seed records.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Verify the seeded citizen NID 5508192841.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>HTTP 200 and alreadyRegistered=true.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>API-005</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Authentication API</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Login accepts valid seeded citizen credentials</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Temporary database is seeded; demo password is demo1234.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>POST the seeded citizen NID and demo password to /api/auth/login.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>HTTP 200, success=true, a token, and a citizen user profile.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>API-006</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Authentication API</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Login rejects an incorrect password</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Temporary database is seeded; no shared account is used.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>POST a seeded citizen NID with an incorrect password.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>HTTP 401 with a credential error and no authentication token.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>API-007</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Authentication API</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Public login blocks an administrator account</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Temporary database is seeded; no shared account is used.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>POST the seeded admin NID and demo password to the public login route.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>HTTP 403 with an access-denied response.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>